<commit_message>
Update skills tracker to reflect current DP-700 exam objectives
Aligns the tracker with the current DP-700 study guide (July 2026).
53 skills, up from 48. Adds 7 new skills, updates 8 renamed ones, moves "Design and implement loading patterns" to domain 1, and fixes a trailing non-breaking space in the domain 1 category name.
</commit_message>
<xml_diff>
--- a/DP700_SkillsMeasured.xlsx
+++ b/DP700_SkillsMeasured.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sh_na\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\WSS Analytics\Conhecimento\DP700\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B9BF677-D85E-4A51-A1AB-F72B829CF38D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{720E8BC2-3C35-4057-84FA-96D5CC21E09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="423" xr2:uid="{197F7256-46D1-4BCD-8146-4714AB14894A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="423" xr2:uid="{197F7256-46D1-4BCD-8146-4714AB14894A}"/>
   </bookViews>
   <sheets>
     <sheet name="DP-700 Study Guide Tracker" sheetId="1" r:id="rId1"/>
@@ -18,30 +18,19 @@
     <sheet name="Learning Path" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DP-700 Study Guide Tracker'!$A$1:$H$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DP-700 Study Guide Tracker'!$A$1:$H$54</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="90">
   <si>
     <t>Design and implement loading patterns</t>
   </si>
@@ -61,12 +50,6 @@
     <t>Choose an appropriate data store</t>
   </si>
   <si>
-    <t>Choose between dataflows, notebooks, and T-SQL for data transformation</t>
-  </si>
-  <si>
-    <t>Create and manage shortcuts to data</t>
-  </si>
-  <si>
     <t>Implement mirroring</t>
   </si>
   <si>
@@ -88,12 +71,6 @@
     <t>Ingest and transform streaming data</t>
   </si>
   <si>
-    <t>Choose an appropriate streaming engine</t>
-  </si>
-  <si>
-    <t>Process data by using eventstreams</t>
-  </si>
-  <si>
     <t>Process data by using Spark structured streaming</t>
   </si>
   <si>
@@ -124,36 +101,21 @@
     <t>Identify and resolve pipeline errors</t>
   </si>
   <si>
-    <t>Identify and resolve dataflow errors</t>
-  </si>
-  <si>
     <t>Identify and resolve notebook errors</t>
   </si>
   <si>
-    <t>Identify and resolve eventhouse errors</t>
-  </si>
-  <si>
-    <t>Identify and resolve eventstream errors</t>
-  </si>
-  <si>
     <t>Identify and resolve T-SQL errors</t>
   </si>
   <si>
     <t>Optimize performance</t>
   </si>
   <si>
-    <t>Optimize a lakehouse table</t>
-  </si>
-  <si>
     <t>Optimize a pipeline</t>
   </si>
   <si>
     <t>Optimize a data warehouse</t>
   </si>
   <si>
-    <t>Optimize eventstreams and eventhouses</t>
-  </si>
-  <si>
     <t>Optimize Spark performance</t>
   </si>
   <si>
@@ -172,9 +134,6 @@
     <t>Configure OneLake workspace settings</t>
   </si>
   <si>
-    <t>Configure data workflow workspace settings</t>
-  </si>
-  <si>
     <t>Implement lifecycle management in Fabric</t>
   </si>
   <si>
@@ -196,9 +155,6 @@
     <t>Implement item-level access controls</t>
   </si>
   <si>
-    <t>Implement row-level, column-level, object-level, and file-level access controls</t>
-  </si>
-  <si>
     <t>Implement dynamic data masking</t>
   </si>
   <si>
@@ -211,9 +167,6 @@
     <t>Orchestrate processes</t>
   </si>
   <si>
-    <t>Choose between a pipeline and a notebook</t>
-  </si>
-  <si>
     <t>Design and implement schedules and event-based triggers</t>
   </si>
   <si>
@@ -241,9 +194,6 @@
     <t>Category</t>
   </si>
   <si>
-    <t>Implement and manage an analytics solution </t>
-  </si>
-  <si>
     <t>Configure Microsoft Fabric workspace settings</t>
   </si>
   <si>
@@ -296,6 +246,60 @@
   </si>
   <si>
     <t>Learning Path URL</t>
+  </si>
+  <si>
+    <t>Configure Spark workspace settings</t>
+  </si>
+  <si>
+    <t>Configure Apache Airflow workspace settings</t>
+  </si>
+  <si>
+    <t>Implement row-level, column-level, object-level, and folder/file-level access controls</t>
+  </si>
+  <si>
+    <t>Implement and use Microsoft Fabric audit logs</t>
+  </si>
+  <si>
+    <t>Configure and implement OneLake security</t>
+  </si>
+  <si>
+    <t>Choose between Dataflow gen 2, a pipeline and a notebook</t>
+  </si>
+  <si>
+    <t>Choose between Dataflows Gen2, notebooks, KQL, and T-SQL for data transformation</t>
+  </si>
+  <si>
+    <t>Create and manage OneLake shortcuts</t>
+  </si>
+  <si>
+    <t>Choose between native tables and OneLake shortcuts in Real-Time Intelligence</t>
+  </si>
+  <si>
+    <t>Choose between Query acceleration for OneLake shortcuts and standard OneLake shortcuts in Real-Time Intelligence</t>
+  </si>
+  <si>
+    <t>Process data by using Eventstreams</t>
+  </si>
+  <si>
+    <t>Identify and resolve Dataflow Gen2 errors</t>
+  </si>
+  <si>
+    <t>Identify and resolve Eventhouse errors</t>
+  </si>
+  <si>
+    <t>Identify and resolve Eventstream errors</t>
+  </si>
+  <si>
+    <t>Identify and resolve OneLake shortcut errors</t>
+  </si>
+  <si>
+    <t>Optimize a Lakehouse table</t>
+  </si>
+  <si>
+    <t>Optimize Eventstreams and Eventhouses</t>
+  </si>
+  <si>
+    <t>Implement and manage an analytics solution</t>
   </si>
 </sst>
 </file>
@@ -327,7 +331,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -337,36 +341,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -396,22 +370,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -422,7 +391,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -460,6 +429,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{922DA8A6-7C8E-4815-A2C9-22A2E8531B8F}" name="Table2" displayName="Table2" ref="A1:B12" totalsRowShown="0">
   <autoFilter ref="A1:B12" xr:uid="{922DA8A6-7C8E-4815-A2C9-22A2E8531B8F}"/>
@@ -477,7 +450,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{549FC1AD-1DC7-4B1B-A35E-39F46AC2C984}" name="Learning Path Key "/>
     <tableColumn id="2" xr3:uid="{12F41F72-848D-40E7-A0D6-30F749D68976}" name="Learning Path Name"/>
-    <tableColumn id="3" xr3:uid="{F0F9991E-66D5-41D8-8021-ADA310D9F924}" name="Learning Path URL" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{F0F9991E-66D5-41D8-8021-ADA310D9F924}" name="Learning Path URL"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -800,600 +773,590 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C00E6A71-0576-4B77-AEC1-148D053D2DA4}">
-  <dimension ref="A1:H49"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H54"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" customWidth="1"/>
-    <col min="2" max="2" width="37.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="4" max="4" width="38.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.26953125" customWidth="1"/>
-    <col min="6" max="6" width="68.90625" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" customWidth="1"/>
-    <col min="8" max="8" width="14.90625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="26.08984375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="2" width="63.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="43.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" customWidth="1"/>
+    <col min="6" max="6" width="68.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="12" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="7" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C2">
         <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C3">
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>42</v>
+      <c r="F3" t="s">
+        <v>32</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C4">
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E4">
         <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
-      <c r="H4" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="E5">
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
-      <c r="H5" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C6">
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
-      <c r="H6" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C7">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E7">
         <v>6</v>
       </c>
       <c r="F7" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
-      <c r="H7" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E8">
         <v>7</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
-      <c r="H8" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C9">
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E9">
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C10">
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E10">
         <v>9</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="G10">
         <v>1</v>
       </c>
-      <c r="H10" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C11">
         <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
-      <c r="H11" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C12">
         <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
-      <c r="H12" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C13">
         <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E13">
         <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
-      <c r="H13" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="E14">
         <v>13</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>56</v>
+      <c r="F14" t="s">
+        <v>43</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
-      <c r="H14" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C15">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="E15">
         <v>14</v>
       </c>
       <c r="F15" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
-      <c r="H15" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="C16">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="E16">
         <v>15</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>58</v>
+      <c r="F16" t="s">
+        <v>76</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
-      <c r="H16" s="4">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="C17">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="E17">
         <v>16</v>
       </c>
       <c r="F17" t="s">
-        <v>1</v>
+        <v>77</v>
       </c>
       <c r="G17">
         <v>1</v>
       </c>
-      <c r="H17" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="C18">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="E18">
         <v>17</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>2</v>
+      <c r="F18" t="s">
+        <v>45</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
-      <c r="H18" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="E19">
         <v>18</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>3</v>
+      <c r="F19" t="s">
+        <v>46</v>
       </c>
       <c r="G19">
         <v>1</v>
       </c>
-      <c r="H19" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H19" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="C20">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E20">
         <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G20">
         <v>1</v>
       </c>
-      <c r="H20" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="C21">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D21" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E21">
         <v>20</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>6</v>
+      <c r="F21" t="s">
+        <v>2</v>
       </c>
       <c r="G21">
         <v>1</v>
       </c>
-      <c r="H21" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H21" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="C22">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E22">
         <v>21</v>
       </c>
-      <c r="F22" s="5" t="s">
-        <v>7</v>
+      <c r="F22" t="s">
+        <v>3</v>
       </c>
       <c r="G22">
         <v>1</v>
       </c>
-      <c r="H22" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="7">
-        <v>2</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="7">
+      <c r="H22" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23">
         <v>22</v>
       </c>
       <c r="D23" t="s">
@@ -1403,21 +1366,21 @@
         <v>22</v>
       </c>
       <c r="F23" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G23">
         <v>1</v>
       </c>
-      <c r="H23" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H23" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C24">
         <v>22</v>
@@ -1428,22 +1391,22 @@
       <c r="E24">
         <v>23</v>
       </c>
-      <c r="F24" s="5" t="s">
-        <v>9</v>
+      <c r="F24" t="s">
+        <v>78</v>
       </c>
       <c r="G24">
         <v>1</v>
       </c>
-      <c r="H24" s="4">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C25">
         <v>22</v>
@@ -1454,24 +1417,24 @@
       <c r="E25">
         <v>24</v>
       </c>
-      <c r="F25" s="5" t="s">
-        <v>10</v>
+      <c r="F25" t="s">
+        <v>79</v>
       </c>
       <c r="G25">
         <v>1</v>
       </c>
-      <c r="H25" s="4">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>2</v>
-      </c>
-      <c r="B26" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26">
+      <c r="H25" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>2</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26" s="2">
         <v>22</v>
       </c>
       <c r="D26" t="s">
@@ -1481,21 +1444,21 @@
         <v>25</v>
       </c>
       <c r="F26" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G26">
-        <v>0.25</v>
-      </c>
-      <c r="H26" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H26" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C27">
         <v>22</v>
@@ -1506,22 +1469,22 @@
       <c r="E27">
         <v>26</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27" s="1">
         <v>12</v>
       </c>
-      <c r="G27">
-        <v>1</v>
-      </c>
-      <c r="H27" s="4">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2</v>
       </c>
       <c r="B28" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C28">
         <v>22</v>
@@ -1532,565 +1495,689 @@
       <c r="E28">
         <v>27</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>13</v>
+      <c r="F28" t="s">
+        <v>8</v>
       </c>
       <c r="G28">
-        <v>0.5</v>
-      </c>
-      <c r="H28" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H28" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C29">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E29">
         <v>28</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>15</v>
+      <c r="F29" t="s">
+        <v>9</v>
       </c>
       <c r="G29">
         <v>1</v>
       </c>
-      <c r="H29" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H29" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C30">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E30">
         <v>29</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>16</v>
+      <c r="F30" t="s">
+        <v>10</v>
       </c>
       <c r="G30">
         <v>1</v>
       </c>
-      <c r="H30" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H30" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2</v>
       </c>
       <c r="B31" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C31">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E31">
         <v>30</v>
       </c>
-      <c r="F31" s="5" t="s">
-        <v>17</v>
+      <c r="F31" t="s">
+        <v>11</v>
       </c>
       <c r="G31">
         <v>1</v>
       </c>
-      <c r="H31" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H31" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C32">
         <v>23</v>
       </c>
       <c r="D32" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E32">
         <v>31</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>18</v>
+      <c r="F32" t="s">
+        <v>80</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
-      <c r="H32" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H32" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C33">
         <v>23</v>
       </c>
       <c r="D33" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E33">
         <v>32</v>
       </c>
-      <c r="F33" s="2" t="s">
-        <v>19</v>
+      <c r="F33" t="s">
+        <v>81</v>
       </c>
       <c r="G33">
         <v>1</v>
       </c>
-      <c r="H33" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H33" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C34">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D34" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E34">
         <v>33</v>
       </c>
       <c r="F34" t="s">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
-      <c r="H34" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H34" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C35">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D35" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E35">
         <v>34</v>
       </c>
       <c r="F35" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="G35">
         <v>1</v>
       </c>
-      <c r="H35" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H35" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C36">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D36" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E36">
         <v>35</v>
       </c>
       <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>2</v>
+      </c>
+      <c r="B37" t="s">
+        <v>31</v>
+      </c>
+      <c r="C37">
         <v>23</v>
       </c>
-      <c r="G36">
-        <v>1</v>
-      </c>
-      <c r="H36" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37">
-        <v>3</v>
-      </c>
-      <c r="B37" t="s">
-        <v>39</v>
-      </c>
-      <c r="C37">
-        <v>31</v>
-      </c>
       <c r="D37" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E37">
         <v>36</v>
       </c>
       <c r="F37" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="G37">
         <v>1</v>
       </c>
-      <c r="H37" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C38">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D38" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E38">
         <v>37</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>26</v>
+      <c r="F38" t="s">
+        <v>17</v>
       </c>
       <c r="G38">
-        <v>0</v>
-      </c>
-      <c r="H38" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H38" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C39">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D39" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E39">
         <v>38</v>
       </c>
-      <c r="F39" s="1" t="s">
-        <v>27</v>
+      <c r="F39" t="s">
+        <v>18</v>
       </c>
       <c r="G39">
-        <v>0</v>
-      </c>
-      <c r="H39" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H39" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>3</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C40">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D40" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E40">
         <v>39</v>
       </c>
-      <c r="F40" s="1" t="s">
-        <v>28</v>
+      <c r="F40" t="s">
+        <v>19</v>
       </c>
       <c r="G40">
-        <v>0</v>
-      </c>
-      <c r="H40" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H40" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>3</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C41">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D41" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E41">
         <v>40</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>29</v>
+      <c r="F41" t="s">
+        <v>20</v>
       </c>
       <c r="G41">
-        <v>0</v>
-      </c>
-      <c r="H41" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H41" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C42">
         <v>32</v>
       </c>
       <c r="D42" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E42">
         <v>41</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>30</v>
+      <c r="F42" t="s">
+        <v>22</v>
       </c>
       <c r="G42">
-        <v>0</v>
-      </c>
-      <c r="H42" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H42" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C43">
         <v>32</v>
       </c>
       <c r="D43" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E43">
         <v>42</v>
       </c>
-      <c r="F43" s="1" t="s">
-        <v>31</v>
+      <c r="F43" t="s">
+        <v>83</v>
       </c>
       <c r="G43">
-        <v>0</v>
-      </c>
-      <c r="H43" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="H43" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C44">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D44" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E44">
         <v>43</v>
       </c>
-      <c r="F44" s="5" t="s">
-        <v>33</v>
+      <c r="F44" t="s">
+        <v>23</v>
       </c>
       <c r="G44">
         <v>1</v>
       </c>
-      <c r="H44" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H44" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C45">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D45" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E45">
         <v>44</v>
       </c>
       <c r="F45" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="G45">
         <v>1</v>
       </c>
-      <c r="H45" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H45" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C46">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D46" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E46">
         <v>45</v>
       </c>
       <c r="F46" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="G46">
         <v>1</v>
       </c>
-      <c r="H46" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H46" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C47">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D47" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E47">
         <v>46</v>
       </c>
-      <c r="F47" s="2" t="s">
-        <v>36</v>
+      <c r="F47" t="s">
+        <v>24</v>
       </c>
       <c r="G47">
         <v>1</v>
       </c>
-      <c r="H47" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H47" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C48">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D48" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E48">
         <v>47</v>
       </c>
-      <c r="F48" s="5" t="s">
-        <v>37</v>
+      <c r="F48" t="s">
+        <v>86</v>
       </c>
       <c r="G48">
         <v>1</v>
       </c>
-      <c r="H48" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C49">
         <v>33</v>
       </c>
       <c r="D49" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E49">
         <v>48</v>
       </c>
       <c r="F49" t="s">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="G49">
-        <v>0.25</v>
-      </c>
-      <c r="H49" s="4">
+        <v>1</v>
+      </c>
+      <c r="H49" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>3</v>
+      </c>
+      <c r="B50" t="s">
+        <v>30</v>
+      </c>
+      <c r="C50">
+        <v>33</v>
+      </c>
+      <c r="D50" t="s">
+        <v>25</v>
+      </c>
+      <c r="E50">
+        <v>49</v>
+      </c>
+      <c r="F50" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50">
+        <v>1</v>
+      </c>
+      <c r="H50" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>3</v>
+      </c>
+      <c r="B51" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51">
+        <v>33</v>
+      </c>
+      <c r="D51" t="s">
+        <v>25</v>
+      </c>
+      <c r="E51">
+        <v>50</v>
+      </c>
+      <c r="F51" t="s">
+        <v>27</v>
+      </c>
+      <c r="G51">
+        <v>1</v>
+      </c>
+      <c r="H51" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>3</v>
+      </c>
+      <c r="B52" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52">
+        <v>33</v>
+      </c>
+      <c r="D52" t="s">
+        <v>25</v>
+      </c>
+      <c r="E52">
+        <v>51</v>
+      </c>
+      <c r="F52" t="s">
+        <v>88</v>
+      </c>
+      <c r="G52">
+        <v>1</v>
+      </c>
+      <c r="H52" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>3</v>
+      </c>
+      <c r="B53" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53">
+        <v>33</v>
+      </c>
+      <c r="D53" t="s">
+        <v>25</v>
+      </c>
+      <c r="E53">
+        <v>52</v>
+      </c>
+      <c r="F53" t="s">
+        <v>28</v>
+      </c>
+      <c r="G53">
+        <v>1</v>
+      </c>
+      <c r="H53" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s">
+        <v>30</v>
+      </c>
+      <c r="C54">
+        <v>33</v>
+      </c>
+      <c r="D54" t="s">
+        <v>25</v>
+      </c>
+      <c r="E54">
+        <v>53</v>
+      </c>
+      <c r="F54" t="s">
+        <v>29</v>
+      </c>
+      <c r="G54">
+        <v>1</v>
+      </c>
+      <c r="H54" s="1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H49" xr:uid="{C00E6A71-0576-4B77-AEC1-148D053D2DA4}"/>
-  <conditionalFormatting sqref="F2:F49">
+  <autoFilter ref="A1:H54" xr:uid="{C00E6A71-0576-4B77-AEC1-148D053D2DA4}"/>
+  <conditionalFormatting sqref="F2:F54">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>AND($G2&gt;0, $G2&lt;1)</formula>
     </cfRule>
@@ -2109,21 +2196,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85E36F6C-F530-445B-8B96-71263B387932}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.26953125" customWidth="1"/>
-    <col min="2" max="2" width="28.26953125" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2131,7 +2218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2139,7 +2226,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2147,7 +2234,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2155,7 +2242,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2163,7 +2250,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0</v>
       </c>
@@ -2171,7 +2258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>12</v>
       </c>
@@ -2179,7 +2266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>12</v>
       </c>
@@ -2187,7 +2274,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>123</v>
       </c>
@@ -2195,7 +2282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>123</v>
       </c>
@@ -2203,7 +2290,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>123</v>
       </c>
@@ -2222,88 +2309,88 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{351084D2-7CF8-432B-B66B-4E53B6E9F1DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="49.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="84.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="84.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>82</v>
+        <v>65</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>